<commit_message>
Fix trailing spaces in Template 4 co-schedule room names
"J-120 " → "J-120" for Guitar Block entries (rows 9-10).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JivS7itntrfpsMmueC8Acs
</commit_message>
<xml_diff>
--- a/templates/Template_4_CoSchedule_Groups.xlsx
+++ b/templates/Template_4_CoSchedule_Groups.xlsx
@@ -1,127 +1,60 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jCiofalo\Desktop\AI MASTER SCHEDULER TEMPLATES 07.31.26\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D13C3900-E4E1-4E55-90F5-A542623863AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30168" windowHeight="19464" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="30168" windowHeight="19464" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Co-Schedule Groups" sheetId="1" r:id="rId1"/>
+    <sheet name="Co-Schedule Groups" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="19">
-  <si>
-    <t>Co-Schedule Group Name</t>
-  </si>
-  <si>
-    <t>Course Code</t>
-  </si>
-  <si>
-    <t>Teacher ID</t>
-  </si>
-  <si>
-    <t>Prescribed Room</t>
-  </si>
-  <si>
-    <t>REQUIRED</t>
-  </si>
-  <si>
-    <t>OPTIONAL</t>
-  </si>
-  <si>
-    <t>J-322</t>
-  </si>
-  <si>
-    <t>Theater Block</t>
-  </si>
-  <si>
-    <t>AP Art Block</t>
-  </si>
-  <si>
-    <t>Italian Block</t>
-  </si>
-  <si>
-    <t>Guitar Block</t>
-  </si>
-  <si>
-    <t>Studio Art Block</t>
-  </si>
-  <si>
-    <t>Programming Block</t>
-  </si>
-  <si>
-    <t>Robotics Block</t>
-  </si>
-  <si>
-    <t>S-237</t>
-  </si>
-  <si>
-    <t xml:space="preserve">J-120 </t>
-  </si>
-  <si>
-    <t>Auditorium</t>
-  </si>
-  <si>
-    <t>J-223</t>
-  </si>
-  <si>
-    <t>S-338</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF375623"/>
       <name val="Arial"/>
       <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF375623"/>
+      <sz val="10"/>
     </font>
     <font>
-      <i/>
-      <sz val="10"/>
-      <color rgb="FF806000"/>
       <name val="Arial"/>
       <family val="2"/>
+      <i val="1"/>
+      <color rgb="FF806000"/>
+      <sz val="10"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -178,39 +111,98 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -498,266 +490,350 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14.44140625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="28.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="4">
+    <row r="1" ht="28.2" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Co-Schedule Group Name</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Course Code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Teacher ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Prescribed Room</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>REQUIRED</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>AP Art Block</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="n">
         <v>253</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="5" t="n">
         <v>105810</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="4">
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>AP Art Block</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
         <v>254</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="5" t="n">
         <v>105810</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="4">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>AP Art Block</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
         <v>255</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="5" t="n">
         <v>105810</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="4">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>AP Art Block</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
         <v>764</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="5" t="n">
         <v>105810</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="6">
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Italian Block</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
         <v>333</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="5" t="n">
         <v>106762</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="6">
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>S-237</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Italian Block</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
         <v>359</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="5" t="n">
         <v>106762</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="6">
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>S-237</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Guitar Block</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
         <v>201</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="5" t="n">
         <v>102255</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="6">
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>J-120</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Guitar Block</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
         <v>203</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="5" t="n">
         <v>102255</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="6">
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>J-120</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Theater Block</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n">
         <v>227</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="5" t="n">
         <v>122002</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6">
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Auditorium</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Theater Block</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n">
         <v>228</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="5" t="n">
         <v>122002</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="6">
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Auditorium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Studio Art Block</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n">
         <v>242</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="5" t="n">
         <v>105810</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="6">
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>Studio Art Block</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
         <v>243</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="5" t="n">
         <v>105810</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="4">
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>J-322</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>Programming Block</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
         <v>473</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="5" t="n">
         <v>106753</v>
       </c>
-      <c r="D15" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="4">
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>J-223</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Programming Block</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="n">
         <v>494</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="5" t="n">
         <v>106753</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="4">
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>J-223</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Robotics Block</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="n">
         <v>590</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="5" t="n">
         <v>117304</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="4">
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>S-338</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>Robotics Block</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
         <v>591</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="5" t="n">
         <v>117304</v>
       </c>
-      <c r="D18" s="4" t="s">
-        <v>18</v>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>S-338</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>